<commit_message>
fix: formatear valores con K/M en graficos y separadores de miles en tablas
</commit_message>
<xml_diff>
--- a/data/Fuentes de datos/Intervenciones de infraestructura/22 SEDES.xlsx
+++ b/data/Fuentes de datos/Intervenciones de infraestructura/22 SEDES.xlsx
@@ -1,23 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26026"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cperez\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jorge\Documents\GOBIERNO_DE_DATOS\Data_Steward\Observatorio_de_Educación\data\Fuentes de datos\Intervenciones de infraestructura\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9553FADF-4791-402B-B742-7719ED43E6ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7530"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja9" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -53,7 +64,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
@@ -405,8 +416,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="D3:M20"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="D1:M18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="16.28515625" customWidth="1"/>
@@ -421,341 +432,341 @@
     <col min="13" max="13" width="14.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1">
+        <v>2025</v>
+      </c>
+      <c r="H1">
+        <v>2026</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="2">
+        <v>2709591630</v>
+      </c>
+      <c r="F2" s="3">
+        <f>+E2/$E$6</f>
+        <v>0.28522017187917914</v>
+      </c>
+      <c r="G2" s="4">
+        <v>945986179</v>
+      </c>
+      <c r="H2" s="5">
+        <v>1619416206</v>
+      </c>
+      <c r="I2" s="5">
+        <f>+G2+H2</f>
+        <v>2565402385</v>
+      </c>
+      <c r="J2" s="5">
+        <f>+E2-I2</f>
+        <v>144189245</v>
+      </c>
+      <c r="K2" s="5"/>
+      <c r="L2" s="4">
+        <f>+ROUND(H14*$G$6,0)</f>
+        <v>963783683</v>
+      </c>
+      <c r="M2" s="4">
+        <f>+G2-L2</f>
+        <v>-17797504</v>
+      </c>
+    </row>
     <row r="3" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D3" t="s">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>2025</v>
-      </c>
-      <c r="H3">
-        <v>2026</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="E3" s="2">
+        <v>2340696555</v>
+      </c>
+      <c r="F3" s="3">
+        <f t="shared" ref="F3:F5" si="0">+E3/$E$6</f>
+        <v>0.24638911131198854</v>
+      </c>
+      <c r="G3" s="4">
+        <v>817195686</v>
+      </c>
+      <c r="H3" s="5">
+        <v>1352474439</v>
+      </c>
+      <c r="I3" s="5">
+        <f>+G3+H3</f>
+        <v>2169670125</v>
+      </c>
+      <c r="J3" s="5">
+        <f>+E3-I3</f>
+        <v>171026430</v>
+      </c>
+      <c r="K3" s="5"/>
+      <c r="L3" s="4">
+        <f t="shared" ref="L3:L5" si="1">+ROUND(H15*$G$6,0)</f>
+        <v>815112934</v>
+      </c>
+      <c r="M3" s="4">
+        <f t="shared" ref="M3:M5" si="2">+G3-L3</f>
+        <v>2082752</v>
       </c>
     </row>
     <row r="4" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E4" s="2">
-        <v>2709591630</v>
+        <v>2282860712</v>
       </c>
       <c r="F4" s="3">
-        <f>+E4/$E$8</f>
-        <v>0.28522017187917914</v>
+        <f t="shared" si="0"/>
+        <v>0.24030112783189592</v>
       </c>
       <c r="G4" s="4">
-        <v>945986179</v>
+        <v>797003747</v>
       </c>
       <c r="H4" s="5">
-        <v>1619416206</v>
+        <v>1247069881</v>
       </c>
       <c r="I4" s="5">
         <f>+G4+H4</f>
-        <v>2565402385</v>
+        <v>2044073628</v>
       </c>
       <c r="J4" s="5">
         <f>+E4-I4</f>
-        <v>144189245</v>
+        <v>238787084</v>
       </c>
       <c r="K4" s="5"/>
       <c r="L4" s="4">
-        <f>+ROUND(H16*$G$8,0)</f>
-        <v>963783683</v>
+        <f t="shared" si="1"/>
+        <v>767928190</v>
       </c>
       <c r="M4" s="4">
-        <f>+G4-L4</f>
-        <v>-17797504</v>
+        <f t="shared" si="2"/>
+        <v>29075557</v>
       </c>
     </row>
     <row r="5" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E5" s="2">
-        <v>2340696555</v>
+        <v>2166851093</v>
       </c>
       <c r="F5" s="3">
-        <f t="shared" ref="F5:F7" si="0">+E5/$E$8</f>
-        <v>0.24638911131198854</v>
+        <f t="shared" si="0"/>
+        <v>0.2280895889769364</v>
       </c>
       <c r="G5" s="4">
-        <v>817195686</v>
+        <v>756501888</v>
       </c>
       <c r="H5" s="5">
-        <v>1352474439</v>
+        <v>1292721005</v>
       </c>
       <c r="I5" s="5">
         <f>+G5+H5</f>
-        <v>2169670125</v>
+        <v>2049222893</v>
       </c>
       <c r="J5" s="5">
         <f>+E5-I5</f>
-        <v>171026430</v>
+        <v>117628200</v>
       </c>
       <c r="K5" s="5"/>
       <c r="L5" s="4">
-        <f t="shared" ref="L5:L7" si="1">+ROUND(H17*$G$8,0)</f>
-        <v>815112934</v>
-      </c>
-      <c r="M5" s="4">
-        <f t="shared" ref="M5:M7" si="2">+G5-L5</f>
-        <v>2082752</v>
-      </c>
-    </row>
-    <row r="6" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="D6" t="s">
-        <v>5</v>
-      </c>
-      <c r="E6" s="2">
-        <v>2282860712</v>
-      </c>
-      <c r="F6" s="3">
-        <f t="shared" si="0"/>
-        <v>0.24030112783189592</v>
-      </c>
-      <c r="G6" s="4">
-        <v>797003747</v>
-      </c>
-      <c r="H6" s="5">
-        <v>1247069881</v>
-      </c>
-      <c r="I6" s="5">
-        <f>+G6+H6</f>
-        <v>2044073628</v>
-      </c>
-      <c r="J6" s="5">
-        <f>+E6-I6</f>
-        <v>238787084</v>
-      </c>
-      <c r="K6" s="5"/>
-      <c r="L6" s="4">
-        <f t="shared" si="1"/>
-        <v>767928190</v>
-      </c>
-      <c r="M6" s="4">
-        <f t="shared" si="2"/>
-        <v>29075557</v>
-      </c>
-    </row>
-    <row r="7" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="D7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" s="2">
-        <v>2166851093</v>
-      </c>
-      <c r="F7" s="3">
-        <f t="shared" si="0"/>
-        <v>0.2280895889769364</v>
-      </c>
-      <c r="G7" s="4">
-        <v>756501888</v>
-      </c>
-      <c r="H7" s="5">
-        <v>1292721005</v>
-      </c>
-      <c r="I7" s="5">
-        <f>+G7+H7</f>
-        <v>2049222893</v>
-      </c>
-      <c r="J7" s="5">
-        <f>+E7-I7</f>
-        <v>117628200</v>
-      </c>
-      <c r="K7" s="5"/>
-      <c r="L7" s="4">
         <f t="shared" si="1"/>
         <v>769862693</v>
       </c>
-      <c r="M7" s="4">
+      <c r="M5" s="4">
         <f t="shared" si="2"/>
         <v>-13360805</v>
       </c>
     </row>
+    <row r="6" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="E6" s="6">
+        <f>SUM(E2:E5)</f>
+        <v>9499999990</v>
+      </c>
+      <c r="G6" s="7">
+        <f>SUM(G2:G5)</f>
+        <v>3316687500</v>
+      </c>
+      <c r="H6" s="7">
+        <f>SUM(H2:H5)</f>
+        <v>5511681531</v>
+      </c>
+      <c r="I6" s="8">
+        <f>+G6+H6</f>
+        <v>8828369031</v>
+      </c>
+      <c r="J6" s="8">
+        <f>SUM(J2:J5)</f>
+        <v>671630959</v>
+      </c>
+    </row>
     <row r="8" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="E8" s="6">
-        <f>SUM(E4:E7)</f>
-        <v>9499999990</v>
-      </c>
-      <c r="G8" s="7">
-        <f>SUM(G4:G7)</f>
-        <v>3316687500</v>
-      </c>
-      <c r="H8" s="7">
-        <f>SUM(H4:H7)</f>
-        <v>5511681531</v>
-      </c>
-      <c r="I8" s="8">
-        <f>+G8+H8</f>
-        <v>8828369031</v>
-      </c>
-      <c r="J8" s="8">
-        <f>SUM(J4:J7)</f>
-        <v>671630959</v>
+      <c r="D8" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8">
+        <v>2025</v>
+      </c>
+      <c r="H8">
+        <v>2026</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E9" s="9">
+        <v>487644278</v>
+      </c>
+      <c r="F9" s="3">
+        <f>+E9/$E$11</f>
+        <v>0.51330976091252878</v>
+      </c>
+      <c r="G9" s="9">
+        <v>170248806.76465729</v>
+      </c>
+      <c r="H9" s="9">
+        <f>+E9-G9</f>
+        <v>317395471.23534274</v>
+      </c>
+      <c r="I9" s="5">
+        <v>487644278</v>
+      </c>
+      <c r="J9" s="9"/>
+      <c r="K9" s="8">
+        <v>610573599</v>
+      </c>
+      <c r="L9" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
+        <v>4</v>
+      </c>
+      <c r="E10" s="9">
+        <v>462355732</v>
+      </c>
+      <c r="F10" s="3">
+        <f>+E10/$E$11</f>
+        <v>0.48669023908747117</v>
+      </c>
+      <c r="G10" s="9">
+        <v>161419943.23534271</v>
+      </c>
+      <c r="H10" s="9">
+        <f>+E10-G10</f>
+        <v>300935788.76465726</v>
+      </c>
+      <c r="I10" s="5">
+        <v>462355732</v>
+      </c>
+      <c r="J10" s="9"/>
+      <c r="K10" s="5">
+        <v>61057360</v>
+      </c>
+      <c r="L10" t="s">
         <v>7</v>
       </c>
-      <c r="G10">
-        <v>2025</v>
-      </c>
-      <c r="H10">
-        <v>2026</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>2</v>
-      </c>
     </row>
     <row r="11" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="D11" t="s">
-        <v>3</v>
-      </c>
       <c r="E11" s="9">
-        <v>487644278</v>
-      </c>
-      <c r="F11" s="3">
-        <f>+E11/$E$13</f>
-        <v>0.51330976091252878</v>
-      </c>
-      <c r="G11" s="9">
-        <v>170248806.76465729</v>
-      </c>
-      <c r="H11" s="9">
-        <f>+E11-G11</f>
-        <v>317395471.23534274</v>
-      </c>
-      <c r="I11" s="5">
-        <v>487644278</v>
-      </c>
-      <c r="J11" s="9"/>
-      <c r="K11" s="8">
-        <v>610573599</v>
-      </c>
-      <c r="L11" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="D12" t="s">
-        <v>4</v>
-      </c>
-      <c r="E12" s="9">
-        <v>462355732</v>
-      </c>
-      <c r="F12" s="3">
-        <f>+E12/$E$13</f>
-        <v>0.48669023908747117</v>
-      </c>
-      <c r="G12" s="9">
-        <v>161419943.23534271</v>
-      </c>
-      <c r="H12" s="9">
-        <f>+E12-G12</f>
-        <v>300935788.76465726</v>
-      </c>
-      <c r="I12" s="5">
-        <v>462355732</v>
-      </c>
-      <c r="J12" s="9"/>
-      <c r="K12" s="5">
-        <v>61057360</v>
-      </c>
-      <c r="L12" t="s">
-        <v>7</v>
+        <f>SUM(E9:E10)</f>
+        <v>950000010</v>
+      </c>
+      <c r="G11" s="10">
+        <f>+G9+G10</f>
+        <v>331668750</v>
+      </c>
+      <c r="H11" s="10">
+        <f>+H9+H10</f>
+        <v>618331260</v>
+      </c>
+      <c r="I11" s="8">
+        <f>SUM(I9:I10)</f>
+        <v>950000010</v>
+      </c>
+      <c r="J11" s="11">
+        <f>+I11/E6</f>
+        <v>0.10000000115789474</v>
       </c>
     </row>
     <row r="13" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="E13" s="9">
-        <f>SUM(E11:E12)</f>
-        <v>950000010</v>
-      </c>
-      <c r="G13" s="10">
-        <f>+G11+G12</f>
-        <v>331668750</v>
-      </c>
-      <c r="H13" s="10">
-        <f>+H11+H12</f>
-        <v>618331260</v>
-      </c>
-      <c r="I13" s="8">
-        <f>SUM(I11:I12)</f>
-        <v>950000010</v>
-      </c>
-      <c r="J13" s="11">
-        <f>+I13/E8</f>
-        <v>0.10000000115789474</v>
-      </c>
+      <c r="G13" s="9"/>
+      <c r="I13" s="9"/>
+    </row>
+    <row r="14" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="G14" s="9">
+        <v>2565402385</v>
+      </c>
+      <c r="H14" s="12">
+        <f>+G14/$G$18</f>
+        <v>0.29058621994525002</v>
+      </c>
+      <c r="I14" s="12">
+        <v>0.28522017187917914</v>
+      </c>
+      <c r="J14" s="13"/>
     </row>
     <row r="15" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="G15" s="9"/>
-      <c r="I15" s="9"/>
+      <c r="G15" s="9">
+        <v>2169670125</v>
+      </c>
+      <c r="H15" s="12">
+        <f t="shared" ref="H15:H17" si="3">+G15/$G$18</f>
+        <v>0.24576114992264192</v>
+      </c>
+      <c r="I15" s="12">
+        <v>0.24638911131198854</v>
+      </c>
+      <c r="J15" s="13"/>
     </row>
     <row r="16" spans="4:13" x14ac:dyDescent="0.25">
       <c r="G16" s="9">
-        <v>2565402385</v>
+        <v>2044073628</v>
       </c>
       <c r="H16" s="12">
-        <f>+G16/$G$20</f>
-        <v>0.29058621994525002</v>
+        <f t="shared" si="3"/>
+        <v>0.23153468333985869</v>
       </c>
       <c r="I16" s="12">
-        <v>0.28522017187917914</v>
+        <v>0.24030112783189592</v>
       </c>
       <c r="J16" s="13"/>
     </row>
     <row r="17" spans="7:10" x14ac:dyDescent="0.25">
       <c r="G17" s="9">
-        <v>2169670125</v>
+        <v>2049222893</v>
       </c>
       <c r="H17" s="12">
-        <f t="shared" ref="H17:H19" si="3">+G17/$G$20</f>
-        <v>0.24576114992264192</v>
-      </c>
-      <c r="I17" s="12">
-        <v>0.24638911131198854</v>
-      </c>
-      <c r="J17" s="13"/>
-    </row>
-    <row r="18" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="G18" s="9">
-        <v>2044073628</v>
-      </c>
-      <c r="H18" s="12">
-        <f t="shared" si="3"/>
-        <v>0.23153468333985869</v>
-      </c>
-      <c r="I18" s="12">
-        <v>0.24030112783189592</v>
-      </c>
-      <c r="J18" s="13"/>
-    </row>
-    <row r="19" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="G19" s="9">
-        <v>2049222893</v>
-      </c>
-      <c r="H19" s="12">
         <f t="shared" si="3"/>
         <v>0.23211794679224937</v>
       </c>
-      <c r="I19" s="12">
+      <c r="I17" s="12">
         <v>0.2280895889769364</v>
       </c>
-      <c r="J19" s="13"/>
-    </row>
-    <row r="20" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="G20" s="10">
-        <f>SUM(G16:G19)</f>
+      <c r="J17" s="13"/>
+    </row>
+    <row r="18" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="G18" s="10">
+        <f>SUM(G14:G17)</f>
         <v>8828369031</v>
       </c>
     </row>

</xml_diff>